<commit_message>
fix minor translation errors
</commit_message>
<xml_diff>
--- a/12_Outcome_measures.xlsx
+++ b/12_Outcome_measures.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\D4YKH4\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wrk\phd\HIS_Forms_for_Stroke_Care\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D57765A-7BEE-4CB6-B24B-B669E5134F28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2E5FE22-30F0-4C95-B122-F46692FED9B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" tabRatio="741" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -232,9 +232,6 @@
     <t>2 points</t>
   </si>
   <si>
-    <t>Deceased</t>
-  </si>
-  <si>
     <t>1 point</t>
   </si>
   <si>
@@ -257,6 +254,9 @@
   </si>
   <si>
     <t>Severe disability; bedridden, incontinent and requiring constant nursing care and attention.</t>
+  </si>
+  <si>
+    <t>Dead</t>
   </si>
 </sst>
 </file>
@@ -370,12 +370,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -383,6 +377,12 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normál" xfId="0" builtinId="0"/>
@@ -714,22 +714,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="9" t="s">
         <v>5</v>
       </c>
     </row>
@@ -746,21 +746,21 @@
       <c r="D2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="7"/>
+      <c r="E2" s="13"/>
       <c r="F2" s="3"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A3" s="8"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
+      <c r="A3" s="11"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
       <c r="D3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="9"/>
+      <c r="E3" s="12"/>
       <c r="F3" s="3"/>
     </row>
     <row r="4" spans="1:6" ht="43.75" x14ac:dyDescent="0.4">
-      <c r="A4" s="8"/>
+      <c r="A4" s="11"/>
       <c r="B4" s="10" t="s">
         <v>10</v>
       </c>
@@ -770,7 +770,7 @@
       <c r="D4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="13" t="s">
         <v>12</v>
       </c>
       <c r="F4" s="6" t="s">
@@ -778,31 +778,31 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
+      <c r="A5" s="11"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
       <c r="D5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="8"/>
+      <c r="E5" s="11"/>
       <c r="F5" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A6" s="8"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
+      <c r="A6" s="11"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="12"/>
       <c r="D6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="9"/>
+      <c r="E6" s="12"/>
       <c r="F6" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="29.15" x14ac:dyDescent="0.4">
-      <c r="A7" s="8"/>
+      <c r="A7" s="11"/>
       <c r="B7" s="10" t="s">
         <v>18</v>
       </c>
@@ -812,7 +812,7 @@
       <c r="D7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="13" t="s">
         <v>12</v>
       </c>
       <c r="F7" s="3" t="s">
@@ -820,43 +820,43 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
+      <c r="A8" s="11"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
       <c r="D8" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="8"/>
+      <c r="E8" s="11"/>
       <c r="F8" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
+      <c r="A9" s="11"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
       <c r="D9" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="8"/>
+      <c r="E9" s="11"/>
       <c r="F9" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A10" s="8"/>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9"/>
+      <c r="A10" s="11"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="12"/>
       <c r="D10" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="9"/>
+      <c r="E10" s="12"/>
       <c r="F10" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="29.15" x14ac:dyDescent="0.4">
-      <c r="A11" s="8"/>
+      <c r="A11" s="11"/>
       <c r="B11" s="10" t="s">
         <v>24</v>
       </c>
@@ -866,7 +866,7 @@
       <c r="D11" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="13" t="s">
         <v>12</v>
       </c>
       <c r="F11" s="3" t="s">
@@ -874,19 +874,19 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A12" s="8"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
+      <c r="A12" s="11"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="12"/>
       <c r="D12" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E12" s="9"/>
+      <c r="E12" s="12"/>
       <c r="F12" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="29.15" x14ac:dyDescent="0.4">
-      <c r="A13" s="8"/>
+      <c r="A13" s="11"/>
       <c r="B13" s="10" t="s">
         <v>27</v>
       </c>
@@ -896,7 +896,7 @@
       <c r="D13" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="13" t="s">
         <v>12</v>
       </c>
       <c r="F13" s="3" t="s">
@@ -904,31 +904,31 @@
       </c>
     </row>
     <row r="14" spans="1:6" ht="29.15" x14ac:dyDescent="0.4">
-      <c r="A14" s="8"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
+      <c r="A14" s="11"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
       <c r="D14" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E14" s="8"/>
+      <c r="E14" s="11"/>
       <c r="F14" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A15" s="8"/>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
+      <c r="A15" s="11"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
       <c r="D15" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E15" s="9"/>
+      <c r="E15" s="12"/>
       <c r="F15" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A16" s="8"/>
+      <c r="A16" s="11"/>
       <c r="B16" s="10" t="s">
         <v>30</v>
       </c>
@@ -938,7 +938,7 @@
       <c r="D16" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="13" t="s">
         <v>12</v>
       </c>
       <c r="F16" s="3" t="s">
@@ -946,19 +946,19 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A17" s="8"/>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9"/>
+      <c r="A17" s="11"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
       <c r="D17" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E17" s="9"/>
+      <c r="E17" s="12"/>
       <c r="F17" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="29.15" x14ac:dyDescent="0.4">
-      <c r="A18" s="8"/>
+      <c r="A18" s="11"/>
       <c r="B18" s="10" t="s">
         <v>33</v>
       </c>
@@ -968,7 +968,7 @@
       <c r="D18" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="13" t="s">
         <v>12</v>
       </c>
       <c r="F18" s="3" t="s">
@@ -976,43 +976,43 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A19" s="8"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
       <c r="D19" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="E19" s="8"/>
+      <c r="E19" s="11"/>
       <c r="F19" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="29.15" x14ac:dyDescent="0.4">
-      <c r="A20" s="8"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
+      <c r="A20" s="11"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
       <c r="D20" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E20" s="8"/>
+      <c r="E20" s="11"/>
       <c r="F20" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A21" s="8"/>
-      <c r="B21" s="9"/>
-      <c r="C21" s="9"/>
+      <c r="A21" s="11"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
       <c r="D21" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="E21" s="9"/>
+      <c r="E21" s="12"/>
       <c r="F21" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A22" s="8"/>
+      <c r="A22" s="11"/>
       <c r="B22" s="10" t="s">
         <v>38</v>
       </c>
@@ -1022,7 +1022,7 @@
       <c r="D22" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="13" t="s">
         <v>12</v>
       </c>
       <c r="F22" s="3" t="s">
@@ -1030,31 +1030,31 @@
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A23" s="8"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
+      <c r="A23" s="11"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
       <c r="D23" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="E23" s="8"/>
+      <c r="E23" s="11"/>
       <c r="F23" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A24" s="8"/>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
+      <c r="A24" s="11"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="12"/>
       <c r="D24" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="E24" s="9"/>
+      <c r="E24" s="12"/>
       <c r="F24" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="29.15" x14ac:dyDescent="0.4">
-      <c r="A25" s="8"/>
+      <c r="A25" s="11"/>
       <c r="B25" s="10" t="s">
         <v>42</v>
       </c>
@@ -1064,7 +1064,7 @@
       <c r="D25" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="E25" s="13" t="s">
         <v>12</v>
       </c>
       <c r="F25" s="3" t="s">
@@ -1072,31 +1072,31 @@
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A26" s="8"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
+      <c r="A26" s="11"/>
+      <c r="B26" s="11"/>
+      <c r="C26" s="11"/>
       <c r="D26" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="E26" s="8"/>
+      <c r="E26" s="11"/>
       <c r="F26" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A27" s="8"/>
-      <c r="B27" s="9"/>
-      <c r="C27" s="9"/>
+      <c r="A27" s="11"/>
+      <c r="B27" s="12"/>
+      <c r="C27" s="12"/>
       <c r="D27" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="E27" s="9"/>
+      <c r="E27" s="12"/>
       <c r="F27" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A28" s="8"/>
+      <c r="A28" s="11"/>
       <c r="B28" s="10" t="s">
         <v>45</v>
       </c>
@@ -1106,7 +1106,7 @@
       <c r="D28" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="E28" s="7" t="s">
+      <c r="E28" s="13" t="s">
         <v>12</v>
       </c>
       <c r="F28" s="3" t="s">
@@ -1114,31 +1114,31 @@
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A29" s="8"/>
-      <c r="B29" s="8"/>
-      <c r="C29" s="8"/>
+      <c r="A29" s="11"/>
+      <c r="B29" s="11"/>
+      <c r="C29" s="11"/>
       <c r="D29" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="E29" s="8"/>
+      <c r="E29" s="11"/>
       <c r="F29" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A30" s="8"/>
-      <c r="B30" s="9"/>
-      <c r="C30" s="9"/>
+      <c r="A30" s="11"/>
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
       <c r="D30" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="E30" s="9"/>
+      <c r="E30" s="12"/>
       <c r="F30" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A31" s="8"/>
+      <c r="A31" s="11"/>
       <c r="B31" s="10" t="s">
         <v>49</v>
       </c>
@@ -1148,7 +1148,7 @@
       <c r="D31" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="E31" s="7" t="s">
+      <c r="E31" s="13" t="s">
         <v>12</v>
       </c>
       <c r="F31" s="3" t="s">
@@ -1156,31 +1156,31 @@
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A32" s="8"/>
-      <c r="B32" s="8"/>
-      <c r="C32" s="8"/>
+      <c r="A32" s="11"/>
+      <c r="B32" s="11"/>
+      <c r="C32" s="11"/>
       <c r="D32" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="E32" s="8"/>
+      <c r="E32" s="11"/>
       <c r="F32" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A33" s="8"/>
-      <c r="B33" s="9"/>
-      <c r="C33" s="9"/>
+      <c r="A33" s="11"/>
+      <c r="B33" s="12"/>
+      <c r="C33" s="12"/>
       <c r="D33" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="E33" s="9"/>
+      <c r="E33" s="12"/>
       <c r="F33" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A34" s="9"/>
+      <c r="A34" s="12"/>
       <c r="B34" s="5" t="s">
         <v>53</v>
       </c>
@@ -1208,187 +1208,213 @@
       <c r="D35" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E35" s="7"/>
+      <c r="E35" s="13"/>
       <c r="F35" s="3" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="29.15" x14ac:dyDescent="0.4">
-      <c r="A36" s="8"/>
-      <c r="B36" s="8"/>
-      <c r="C36" s="8"/>
+      <c r="A36" s="11"/>
+      <c r="B36" s="11"/>
+      <c r="C36" s="11"/>
       <c r="D36" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="E36" s="8"/>
+      <c r="E36" s="11"/>
       <c r="F36" s="3" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="29.15" x14ac:dyDescent="0.4">
-      <c r="A37" s="8"/>
-      <c r="B37" s="8"/>
-      <c r="C37" s="8"/>
+      <c r="A37" s="11"/>
+      <c r="B37" s="11"/>
+      <c r="C37" s="11"/>
       <c r="D37" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E37" s="8"/>
+      <c r="E37" s="11"/>
       <c r="F37" s="3" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A38" s="8"/>
-      <c r="B38" s="8"/>
-      <c r="C38" s="8"/>
+      <c r="A38" s="11"/>
+      <c r="B38" s="11"/>
+      <c r="C38" s="11"/>
       <c r="D38" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="E38" s="8"/>
+      <c r="E38" s="11"/>
       <c r="F38" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="29.15" x14ac:dyDescent="0.4">
-      <c r="A39" s="8"/>
-      <c r="B39" s="8"/>
-      <c r="C39" s="8"/>
+      <c r="A39" s="11"/>
+      <c r="B39" s="11"/>
+      <c r="C39" s="11"/>
       <c r="D39" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="E39" s="8"/>
+      <c r="E39" s="11"/>
       <c r="F39" s="3" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A40" s="8"/>
-      <c r="B40" s="8"/>
-      <c r="C40" s="8"/>
+      <c r="A40" s="11"/>
+      <c r="B40" s="11"/>
+      <c r="C40" s="11"/>
       <c r="D40" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="E40" s="8"/>
+      <c r="E40" s="11"/>
       <c r="F40" s="3" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A41" s="8"/>
-      <c r="B41" s="8"/>
-      <c r="C41" s="8"/>
+      <c r="A41" s="11"/>
+      <c r="B41" s="11"/>
+      <c r="C41" s="11"/>
       <c r="D41" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="E41" s="8"/>
+      <c r="E41" s="11"/>
       <c r="F41" s="3" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A42" s="9"/>
-      <c r="B42" s="9"/>
-      <c r="C42" s="9"/>
+      <c r="A42" s="12"/>
+      <c r="B42" s="12"/>
+      <c r="C42" s="12"/>
       <c r="D42" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E42" s="12"/>
+      <c r="F42" s="3" t="s">
         <v>70</v>
-      </c>
-      <c r="E42" s="9"/>
-      <c r="F42" s="3" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A43" s="10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C43" s="10" t="s">
         <v>7</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="E43" s="7"/>
+        <v>72</v>
+      </c>
+      <c r="E43" s="13"/>
       <c r="F43" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A44" s="8"/>
-      <c r="B44" s="8"/>
-      <c r="C44" s="8"/>
+      <c r="A44" s="11"/>
+      <c r="B44" s="11"/>
+      <c r="C44" s="11"/>
       <c r="D44" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E44" s="11"/>
+      <c r="F44" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="29.15" x14ac:dyDescent="0.4">
+      <c r="A45" s="11"/>
+      <c r="B45" s="11"/>
+      <c r="C45" s="11"/>
+      <c r="D45" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="E44" s="8"/>
-      <c r="F44" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="29.15" x14ac:dyDescent="0.4">
-      <c r="A45" s="8"/>
-      <c r="B45" s="8"/>
-      <c r="C45" s="8"/>
-      <c r="D45" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E45" s="8"/>
+      <c r="E45" s="11"/>
       <c r="F45" s="3" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A46" s="8"/>
-      <c r="B46" s="8"/>
-      <c r="C46" s="8"/>
+      <c r="A46" s="11"/>
+      <c r="B46" s="11"/>
+      <c r="C46" s="11"/>
       <c r="D46" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="E46" s="8"/>
+        <v>75</v>
+      </c>
+      <c r="E46" s="11"/>
       <c r="F46" s="3" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="29.15" x14ac:dyDescent="0.4">
-      <c r="A47" s="8"/>
-      <c r="B47" s="8"/>
-      <c r="C47" s="8"/>
+      <c r="A47" s="11"/>
+      <c r="B47" s="11"/>
+      <c r="C47" s="11"/>
       <c r="D47" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E47" s="8"/>
+        <v>76</v>
+      </c>
+      <c r="E47" s="11"/>
       <c r="F47" s="3" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A48" s="8"/>
-      <c r="B48" s="8"/>
-      <c r="C48" s="8"/>
+      <c r="A48" s="11"/>
+      <c r="B48" s="11"/>
+      <c r="C48" s="11"/>
       <c r="D48" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="E48" s="8"/>
+        <v>77</v>
+      </c>
+      <c r="E48" s="11"/>
       <c r="F48" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A49" s="9"/>
-      <c r="B49" s="9"/>
-      <c r="C49" s="9"/>
+      <c r="A49" s="12"/>
+      <c r="B49" s="12"/>
+      <c r="C49" s="12"/>
       <c r="D49" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="E49" s="9"/>
+        <v>78</v>
+      </c>
+      <c r="E49" s="12"/>
       <c r="F49" s="3" t="s">
         <v>62</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="42">
+    <mergeCell ref="E18:E21"/>
+    <mergeCell ref="A35:A42"/>
+    <mergeCell ref="B35:B42"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="A2:A34"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="C22:C24"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="C18:C21"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="E22:E24"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="C43:C49"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="C35:C42"/>
+    <mergeCell ref="E25:E27"/>
+    <mergeCell ref="C28:C30"/>
+    <mergeCell ref="B25:B27"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="E35:E42"/>
     <mergeCell ref="A43:A49"/>
     <mergeCell ref="E43:E49"/>
     <mergeCell ref="E4:E6"/>
@@ -1405,32 +1431,6 @@
     <mergeCell ref="B13:B15"/>
     <mergeCell ref="B16:B17"/>
     <mergeCell ref="B7:B10"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="E22:E24"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="C43:C49"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="C35:C42"/>
-    <mergeCell ref="E25:E27"/>
-    <mergeCell ref="C28:C30"/>
-    <mergeCell ref="B25:B27"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="B22:B24"/>
-    <mergeCell ref="E35:E42"/>
-    <mergeCell ref="E18:E21"/>
-    <mergeCell ref="A35:A42"/>
-    <mergeCell ref="B35:B42"/>
-    <mergeCell ref="B18:B21"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="A2:A34"/>
-    <mergeCell ref="B31:B33"/>
-    <mergeCell ref="C22:C24"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="C18:C21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>